<commit_message>
implemented visualization and health check
</commit_message>
<xml_diff>
--- a/evaluations/results/EXECUTIVE_PERFORMANCE_REPORT_V10.xlsx
+++ b/evaluations/results/EXECUTIVE_PERFORMANCE_REPORT_V10.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/himanth/PCB/main_ST_AI/Main/AI-Enabled-Ticketing-System-main 6/evaluations/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{326E28A9-C0D2-ED4D-85D0-A0B7A1AF5958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD9854E4-B556-1F4E-91DE-FA0D60FA8A5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1_FULL_BENCHMARK_DATA" sheetId="1" r:id="rId1"/>
@@ -1103,12 +1103,6 @@
     <t>The values represent actual production consumption per ticket. Input includes user query + RAG context window; Output is the bot's generated response.</t>
   </si>
   <si>
-    <t>OCI Context Capacity: 128k+ Tokens | Configured Max Output: 6,000 Tokens</t>
-  </si>
-  <si>
-    <t>OCI Context Capacity: 128k+ Tokens | Configured Max Output: 600 Tokens</t>
-  </si>
-  <si>
     <t>METRIC</t>
   </si>
   <si>
@@ -1185,6 +1179,12 @@
   </si>
   <si>
     <t>Fastest response time for real-time support.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Configured Max Output: 6,000 Tokens</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Configured Max Output: 600 Tokens</t>
   </si>
 </sst>
 </file>
@@ -8103,7 +8103,7 @@
         <v>23</v>
       </c>
       <c r="B31" t="s">
-        <v>225</v>
+        <v>251</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
@@ -8111,7 +8111,7 @@
         <v>60</v>
       </c>
       <c r="B32" t="s">
-        <v>226</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -8132,100 +8132,100 @@
   <sheetData>
     <row r="1" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>228</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="B2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C2" t="s">
         <v>231</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>232</v>
-      </c>
-      <c r="C2" t="s">
-        <v>233</v>
-      </c>
-      <c r="D2" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B3" t="s">
+        <v>234</v>
+      </c>
+      <c r="C3" t="s">
         <v>235</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>236</v>
-      </c>
-      <c r="C3" t="s">
-        <v>237</v>
-      </c>
-      <c r="D3" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B4" t="s">
+        <v>238</v>
+      </c>
+      <c r="C4" t="s">
         <v>239</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
         <v>240</v>
-      </c>
-      <c r="C4" t="s">
-        <v>241</v>
-      </c>
-      <c r="D4" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C5" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="D5" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B6" t="s">
+        <v>244</v>
+      </c>
+      <c r="C6" t="s">
         <v>245</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
         <v>246</v>
-      </c>
-      <c r="C6" t="s">
-        <v>247</v>
-      </c>
-      <c r="D6" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B7" t="s">
+        <v>248</v>
+      </c>
+      <c r="C7" t="s">
         <v>249</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
         <v>250</v>
-      </c>
-      <c r="C7" t="s">
-        <v>251</v>
-      </c>
-      <c r="D7" t="s">
-        <v>252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added fallback model and recursive learning response
</commit_message>
<xml_diff>
--- a/evaluations/results/EXECUTIVE_PERFORMANCE_REPORT_V10.xlsx
+++ b/evaluations/results/EXECUTIVE_PERFORMANCE_REPORT_V10.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/himanth/PCB/main_ST_AI/Main/AI-Enabled-Ticketing-System-main 6/evaluations/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD9854E4-B556-1F4E-91DE-FA0D60FA8A5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D401E5D4-D6CA-D944-8CD9-1DA07D8CFC08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1_FULL_BENCHMARK_DATA" sheetId="1" r:id="rId1"/>
@@ -1594,7 +1594,9 @@
     <col min="15" max="15" width="14" customWidth="1"/>
     <col min="16" max="16" width="15" customWidth="1"/>
     <col min="17" max="18" width="14" customWidth="1"/>
-    <col min="19" max="22" width="40" customWidth="1"/>
+    <col min="19" max="20" width="40" customWidth="1"/>
+    <col min="21" max="21" width="79.83203125" customWidth="1"/>
+    <col min="22" max="22" width="40" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="16" x14ac:dyDescent="0.2">

</xml_diff>